<commit_message>
building_type -> dwelling_type rename pbl file
</commit_message>
<xml_diff>
--- a/data_households_PBL_2023.xlsx
+++ b/data_households_PBL_2023.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AteHe\Desktop\Modellen\data_Generic\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FFCD031-85B9-4B10-9BE8-AD299CB9BB2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A384C43-60A7-49EA-8C58-70CA165B6B27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{C7D0C498-E103-47AD-98B6-0A7C94B1B2AA}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{C7D0C498-E103-47AD-98B6-0A7C94B1B2AA}"/>
   </bookViews>
   <sheets>
     <sheet name="info" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3237" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3238" uniqueCount="78">
   <si>
     <t xml:space="preserve">Data based on PBL referentieverbruik </t>
   </si>
@@ -242,9 +242,6 @@
     <t>x</t>
   </si>
   <si>
-    <t>building_type</t>
-  </si>
-  <si>
     <t>ownership_type</t>
   </si>
   <si>
@@ -273,6 +270,12 @@
   </si>
   <si>
     <t>constant_space_heating_gas_m3pa</t>
+  </si>
+  <si>
+    <t>dwelling_type</t>
+  </si>
+  <si>
+    <t>(dwelling_type)</t>
   </si>
 </sst>
 </file>
@@ -679,8 +682,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9355E6FB-0B67-43A6-BE59-37B53E92A2EF}">
-  <dimension ref="A1:B67"/>
+  <dimension ref="A1:D67"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="4" max="4" width="13.7265625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
@@ -737,7 +743,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="3">
         <v>0</v>
       </c>
@@ -745,7 +751,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="3">
         <v>1</v>
       </c>
@@ -753,7 +759,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="3">
         <v>2</v>
       </c>
@@ -761,7 +767,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="3">
         <v>3</v>
       </c>
@@ -769,7 +775,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" s="3">
         <v>4</v>
       </c>
@@ -777,7 +783,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="3">
         <v>5</v>
       </c>
@@ -785,7 +791,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="3">
         <v>6</v>
       </c>
@@ -793,7 +799,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" s="3">
         <v>7</v>
       </c>
@@ -801,7 +807,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" s="3">
         <v>8</v>
       </c>
@@ -809,7 +815,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" s="3">
         <v>9</v>
       </c>
@@ -817,7 +823,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" s="3">
         <v>10</v>
       </c>
@@ -825,7 +831,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="3">
         <v>11</v>
       </c>
@@ -833,12 +839,15 @@
         <v>22</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="D30" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" s="3">
         <v>1</v>
       </c>
@@ -846,7 +855,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" s="3">
         <v>2</v>
       </c>
@@ -1073,25 +1082,25 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" t="s">
         <v>66</v>
       </c>
-      <c r="B1" t="s">
-        <v>69</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>67</v>
       </c>
-      <c r="D1" t="s">
-        <v>68</v>
-      </c>
       <c r="E1" t="s">
+        <v>73</v>
+      </c>
+      <c r="F1" t="s">
         <v>74</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>75</v>
-      </c>
-      <c r="G1" t="s">
-        <v>76</v>
       </c>
       <c r="H1" t="s">
         <v>55</v>
@@ -92973,7 +92982,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I3169" xr:uid="{CDEE166B-95A0-4C32-BF8B-7DA03C5AB730}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -92992,19 +93000,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B1" t="s">
         <v>69</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>70</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>71</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>72</v>
-      </c>
-      <c r="E1" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">

</xml_diff>